<commit_message>
Add US100 and BTCUSD as extra pairs in simple tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXLbN52gNPv6MZpUt65Vuj
</commit_message>
<xml_diff>
--- a/KLR_Simple_Tracker.xlsx
+++ b/KLR_Simple_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="92">
   <si>
     <t xml:space="preserve">MY TRADING RULES</t>
   </si>
@@ -97,7 +97,7 @@
     <t xml:space="preserve">Pairs</t>
   </si>
   <si>
-    <t xml:space="preserve">XAUUSD, EURUSD, GBPUSD, GER40, US500. Nothing else.</t>
+    <t xml:space="preserve">Main: XAUUSD, EURUSD, GBPUSD, GER40, US500. Extras: US100, BTCUSD. Nothing else.</t>
   </si>
   <si>
     <t xml:space="preserve">Never</t>
@@ -190,16 +190,28 @@
     <t xml:space="preserve">1 point = $1 per lot at many brokers. CHECK in MT5.</t>
   </si>
   <si>
+    <t xml:space="preserve">US100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extra. 1 point = $1 per lot at many brokers. CHECK in MT5.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Account</t>
   </si>
   <si>
+    <t xml:space="preserve">BTCUSD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extra. $1 move = $1 per lot (1 BTC contract). CHECK in MT5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk per trade ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.5% of starting balance. Change it on the Trade Log tab.)</t>
+  </si>
+  <si>
     <t xml:space="preserve">In MT5: right-click the pair &gt; Specification. Check the contract size; change the $ value if yours is different.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risk per trade ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.5% of starting balance. Change it on the Trade Log tab.)</t>
   </si>
   <si>
     <t xml:space="preserve">TRADE LOG</t>
@@ -1120,7 +1132,7 @@
         <v>36</v>
       </c>
       <c r="B9" s="9" t="n">
-        <f aca="false">IFERROR(ROUND(ABS(B5-B6)/VLOOKUP(B4,$D$19:$F$23,2,FALSE()),1),"")</f>
+        <f aca="false">IFERROR(ROUND(ABS(B5-B6)/VLOOKUP(B4,$D$19:$F$25,2,FALSE()),1),"")</f>
         <v>30</v>
       </c>
     </row>
@@ -1138,7 +1150,7 @@
         <v>38</v>
       </c>
       <c r="B11" s="12" t="n">
-        <f aca="false">IFERROR(ROUNDDOWN(B10/(B9*VLOOKUP(B4,$D$19:$F$23,3,FALSE())),2),"")</f>
+        <f aca="false">IFERROR(ROUNDDOWN(B10/(B9*VLOOKUP(B4,$D$19:$F$25,3,FALSE())),2),"")</f>
         <v>0.16</v>
       </c>
       <c r="C11" s="4" t="s">
@@ -1159,7 +1171,7 @@
         <v>41</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">IFERROR(B11*B9*1.5*VLOOKUP(B4,$D$19:$F$23,3,FALSE()),"")</f>
+        <f aca="false">IFERROR(B11*B9*1.5*VLOOKUP(B4,$D$19:$F$25,3,FALSE()),"")</f>
         <v>72</v>
       </c>
     </row>
@@ -1257,17 +1269,40 @@
         <v>54</v>
       </c>
     </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D24" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="19" t="s">
+        <v>56</v>
+      </c>
+    </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="19" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B26" s="10" t="n">
         <f aca="false">'Trade Log'!$M$2*'Trade Log'!$M$3</f>
@@ -1276,13 +1311,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>58</v>
+        <v>61</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B4" type="list">
-      <formula1>$D$19:$D$23</formula1>
+      <formula1>$D$19:$D$25</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1319,12 +1357,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L2" s="11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="M2" s="20" t="n">
         <v>10000</v>
@@ -1332,10 +1370,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="M3" s="21" t="n">
         <v>0.005</v>
@@ -1343,10 +1381,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M4" s="22" t="n">
         <f aca="false">M2+SUM(J7:J206)</f>
@@ -1355,40 +1393,40 @@
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E6" s="16" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="I6" s="16" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7202,7 +7240,7 @@
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7:B206" type="list">
-      <formula1>Calculator!$D$19:$D$23</formula1>
+      <formula1>Calculator!$D$19:$D$25</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K7:K206" type="list">
@@ -7225,7 +7263,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -7235,12 +7273,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B3" s="28" t="n">
         <f aca="false">COUNT('Trade Log'!I7:I206)</f>
@@ -7249,7 +7287,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="27" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B4" s="28" t="n">
         <f aca="false">COUNTIF('Trade Log'!H7:H206,"WIN")</f>
@@ -7258,7 +7296,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B5" s="28" t="n">
         <f aca="false">COUNTIF('Trade Log'!H7:H206,"LOSS")</f>
@@ -7267,7 +7305,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B6" s="29" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
@@ -7276,7 +7314,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B7" s="30" t="n">
         <f aca="false">SUM('Trade Log'!I7:I206)</f>
@@ -7285,7 +7323,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B8" s="30" t="n">
         <f aca="false">IFERROR(B7/B3,0)</f>
@@ -7294,7 +7332,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">IFERROR(COUNTIF('Trade Log'!K7:K206,"Yes")/B3,0)</f>
@@ -7303,7 +7341,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B10" s="31" t="n">
         <f aca="false">SUM('Trade Log'!J7:J206)</f>
@@ -7312,7 +7350,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">'Trade Log'!M4</f>
@@ -7321,7 +7359,7 @@
     </row>
     <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7336,12 +7374,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7349,10 +7387,10 @@
         <v>31</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7417,6 +7455,32 @@
       </c>
       <c r="C24" s="24" t="n">
         <f aca="false">SUMIF('Trade Log'!B7:B206,A24,'Trade Log'!I7:I206)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" s="34" t="n">
+        <f aca="false">COUNTIFS('Trade Log'!B7:B206,A25,'Trade Log'!I7:I206,"&gt;-99")</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="24" t="n">
+        <f aca="false">SUMIF('Trade Log'!B7:B206,A25,'Trade Log'!I7:I206)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="34" t="n">
+        <f aca="false">COUNTIFS('Trade Log'!B7:B206,A26,'Trade Log'!I7:I206,"&gt;-99")</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="24" t="n">
+        <f aca="false">SUMIF('Trade Log'!B7:B206,A26,'Trade Log'!I7:I206)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Rules: CHoCH close entry with market order (option A)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXLbN52gNPv6MZpUt65Vuj
</commit_message>
<xml_diff>
--- a/KLR_Simple_Tracker.xlsx
+++ b/KLR_Simple_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="96">
   <si>
     <t xml:space="preserve">MY TRADING RULES</t>
   </si>
@@ -49,13 +49,19 @@
     <t xml:space="preserve">Step 2</t>
   </si>
   <si>
-    <t xml:space="preserve">On the 1-minute chart, price stops going up (or down) and starts turning.</t>
+    <t xml:space="preserve">On the 1-minute chart, mark the last swing of that run (last higher low if it ran up, last lower high if it ran down).</t>
   </si>
   <si>
     <t xml:space="preserve">Step 3</t>
   </si>
   <si>
-    <t xml:space="preserve">One strong candle in the new direction. Enter when price breaks that candle.</t>
+    <t xml:space="preserve">CHoCH: wait for a candle to CLOSE beyond that swing point.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market order as soon as that CHoCH candle closes. No waiting for a retest.</t>
   </si>
   <si>
     <t xml:space="preserve">Stop</t>
@@ -248,9 +254,6 @@
   </si>
   <si>
     <t xml:space="preserve">Buy / Sell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entry</t>
   </si>
   <si>
     <t xml:space="preserve">Target (auto)</t>
@@ -946,7 +949,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -1068,6 +1071,14 @@
       </c>
       <c r="B16" s="3" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1100,25 +1111,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>2650</v>
@@ -1126,7 +1137,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>2647</v>
@@ -1134,7 +1145,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B8" s="8" t="str">
         <f aca="false">IF(OR(B5="",B6="",B5=B6),"",IF(B6&lt;B5,"BUY","SELL"))</f>
@@ -1143,7 +1154,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">IFERROR(ROUND(ABS(B5-B6)/VLOOKUP(B4,$D$19:$H$25,2,FALSE()),1),"")</f>
@@ -1152,7 +1163,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">B27</f>
@@ -1161,19 +1172,19 @@
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">IFERROR(IF(B10/(B9*VLOOKUP(B4,$D$19:$H$25,3,FALSE()))&lt;VLOOKUP(B4,$D$19:$H$25,4,FALSE()),"SKIP",ROUNDDOWN(B10/(B9*VLOOKUP(B4,$D$19:$H$25,3,FALSE()))/VLOOKUP(B4,$D$19:$H$25,5,FALSE())+0.000001,0)*VLOOKUP(B4,$D$19:$H$25,5,FALSE())),"")</f>
         <v>0.16</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B12" s="13" t="n">
         <f aca="false">IF(B8="","",IF(B8="BUY",B5+1.5*(B5-B6),B5-1.5*(B6-B5)))</f>
@@ -1182,7 +1193,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">IFERROR(B11*B9*1.5*VLOOKUP(B4,$D$19:$H$25,3,FALSE()),"")</f>
@@ -1191,7 +1202,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B14" s="10" t="n">
         <f aca="false">IFERROR(B11*B9*VLOOKUP(B4,$D$19:$H$25,3,FALSE()),"")</f>
@@ -1200,40 +1211,40 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D18" s="17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D19" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E19" s="18" t="n">
         <v>0.1</v>
@@ -1248,12 +1259,12 @@
         <v>0.01</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D20" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E20" s="18" t="n">
         <v>0.0001</v>
@@ -1268,12 +1279,12 @@
         <v>0.01</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D21" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E21" s="18" t="n">
         <v>0.0001</v>
@@ -1288,12 +1299,12 @@
         <v>0.01</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D22" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E22" s="18" t="n">
         <v>1</v>
@@ -1308,12 +1319,12 @@
         <v>0.1</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D23" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E23" s="18" t="n">
         <v>1</v>
@@ -1328,12 +1339,12 @@
         <v>0.1</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D24" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E24" s="18" t="n">
         <v>1</v>
@@ -1348,12 +1359,12 @@
         <v>0.1</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D25" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E25" s="18" t="n">
         <v>1</v>
@@ -1368,29 +1379,29 @@
         <v>0.01</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B27" s="10" t="n">
         <f aca="false">'Trade Log'!$M$2*'Trade Log'!$M$3</f>
         <v>50</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1433,12 +1444,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L2" s="11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="M2" s="21" t="n">
         <v>10000</v>
@@ -1446,10 +1457,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="M3" s="22" t="n">
         <v>0.005</v>
@@ -1457,10 +1468,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="M4" s="23" t="n">
         <f aca="false">M2+SUM(J7:J206)</f>
@@ -1469,40 +1480,40 @@
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I6" s="17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L6" s="17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7349,12 +7360,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B3" s="29" t="n">
         <f aca="false">COUNT('Trade Log'!I7:I206)</f>
@@ -7363,7 +7374,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" s="29" t="n">
         <f aca="false">COUNTIF('Trade Log'!H7:H206,"WIN")</f>
@@ -7372,7 +7383,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B5" s="29" t="n">
         <f aca="false">COUNTIF('Trade Log'!H7:H206,"LOSS")</f>
@@ -7381,7 +7392,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B6" s="30" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
@@ -7390,7 +7401,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B7" s="31" t="n">
         <f aca="false">SUM('Trade Log'!I7:I206)</f>
@@ -7399,7 +7410,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B8" s="31" t="n">
         <f aca="false">IFERROR(B7/B3,0)</f>
@@ -7408,7 +7419,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B9" s="30" t="n">
         <f aca="false">IFERROR(COUNTIF('Trade Log'!K7:K206,"Yes")/B3,0)</f>
@@ -7417,7 +7428,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B10" s="32" t="n">
         <f aca="false">SUM('Trade Log'!J7:J206)</f>
@@ -7426,7 +7437,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B11" s="23" t="n">
         <f aca="false">'Trade Log'!M4</f>
@@ -7435,7 +7446,7 @@
     </row>
     <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="33" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7450,28 +7461,28 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B20" s="35" t="n">
         <f aca="false">COUNTIFS('Trade Log'!B7:B206,A20,'Trade Log'!I7:I206,"&gt;-99")</f>
@@ -7484,7 +7495,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B21" s="35" t="n">
         <f aca="false">COUNTIFS('Trade Log'!B7:B206,A21,'Trade Log'!I7:I206,"&gt;-99")</f>
@@ -7497,7 +7508,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B22" s="35" t="n">
         <f aca="false">COUNTIFS('Trade Log'!B7:B206,A22,'Trade Log'!I7:I206,"&gt;-99")</f>
@@ -7510,7 +7521,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B23" s="35" t="n">
         <f aca="false">COUNTIFS('Trade Log'!B7:B206,A23,'Trade Log'!I7:I206,"&gt;-99")</f>
@@ -7523,7 +7534,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B24" s="35" t="n">
         <f aca="false">COUNTIFS('Trade Log'!B7:B206,A24,'Trade Log'!I7:I206,"&gt;-99")</f>
@@ -7536,7 +7547,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B25" s="35" t="n">
         <f aca="false">COUNTIFS('Trade Log'!B7:B206,A25,'Trade Log'!I7:I206,"&gt;-99")</f>
@@ -7549,7 +7560,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B26" s="35" t="n">
         <f aca="false">COUNTIFS('Trade Log'!B7:B206,A26,'Trade Log'!I7:I206,"&gt;-99")</f>

</xml_diff>